<commit_message>
Monitor Excel changes and trigger validated approval.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D17E9608-D004-4566-AC1B-A045EA419917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE75DD6-F97F-4C93-9947-E33B18596F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3190" yWindow="2810" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Add validated publishing, file monitoring, and Power BI UI discovery.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE75DD6-F97F-4C93-9947-E33B18596F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6B7C23-2BFC-4EA2-BDB8-BBAD1E902C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3190" yWindow="2810" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="1" r:id="rId1"/>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>500000</v>
+        <v>510000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>

<commit_message>
Add experimental Power BI refresh trigger.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6B7C23-2BFC-4EA2-BDB8-BBAD1E902C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C891EB-8C6B-47A4-8A68-D533E93C553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>510000</v>
+        <v>500000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>

<commit_message>
Trigger experimental Power BI refresh after validated approval.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C891EB-8C6B-47A4-8A68-D533E93C553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5997563D-92C5-4B58-95DB-10437C2B1738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>500000</v>
+        <v>510000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>

<commit_message>
Guard monitored refresh with timestamp retries and uncertain-outcome stops.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A490E0AA-1DCA-4018-8804-7425B921011A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7183D714-0EFB-4261-B738-639064B5F523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>500000</v>
+        <v>510000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>

<commit_message>
Add monitoring controls and cooperative stop to desktop UI.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F50FBE-DCF5-4834-AA9D-1F15610E56AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFAF2AA-8DCD-4DE2-ACC0-E6CFCCDEFC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>500000</v>
+        <v>510000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>

<commit_message>
Add desktop UI with monitoring controls and cooperative stop.
</commit_message>
<xml_diff>
--- a/data/approved/FlowBI_Project_Management.xlsx
+++ b/data/approved/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB40E421-BF95-43BE-A0A9-1F9A2AEDBE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041B28A3-AA5D-4715-9D84-91748476C73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>510000</v>
+        <v>500000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>